<commit_message>
v1.30 - GPS tracker avanzato con IndexedDB buffer offline, batch Firestore, heartbeat, retry automatico e rimozione Google Sheets
</commit_message>
<xml_diff>
--- a/dati/GESTIONE.xlsx
+++ b/dati/GESTIONE.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Il mio Drive\AppLogSolution\dati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14EFC9C-555C-41CC-AF28-5AF746CDB16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E75B24A-D18D-4AE2-8DF5-363DFDCD226D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26480" yWindow="850" windowWidth="19200" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
+    <sheet name="Registro" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="v1jhr7aIR2bLfDJSDHV/Eav7EaERU9NJD7+dOEa2O4M="/>

</xml_diff>